<commit_message>
Lat and Long as separate fields, and what did you find now multi check box and conditional on an inspection
</commit_message>
<xml_diff>
--- a/goanna_burrow_detection.xlsx
+++ b/goanna_burrow_detection.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -448,248 +448,301 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>hint</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>relevant</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>location_lat</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>GPS latitude</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>location_lon</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>GPS longitude</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>GPS coordinates or place name</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>hunting_team_names</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hunting team member names</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>start_time</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Start time</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>record_number</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Record number</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>duration_seconds</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Duration (seconds)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Time taken to find the burrow</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>people_searching</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Number of people searching</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>select_one dig_or_inspect_choices</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>dig_or_inspect</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Was the burrow dug or just inspected?</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>select_multiple found_choices</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>what_did_you_find</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>What did you find?</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>${dig_or_inspect} = 'Yes'</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>hunting_team_names</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Hunting team member names</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>time</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>start_time</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Start time</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>record_number</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Record number</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>duration_seconds</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Duration (seconds)</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Time taken to find the burrow</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>people_searching</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Number of people searching</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>select_one dig_or_inspect_choices</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>dig_or_inspect</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Was the burrow dug or just inspected?</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>what_did_you_find</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>What was found</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>e.g. goanna, eggs, empty burrow</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>what_did_you_find_other</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Please specify</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>no</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>selected(${what_did_you_find}, 'other')</t>
         </is>
       </c>
     </row>
@@ -704,7 +757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -713,53 +766,138 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>list_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>dig_or_inspect_choices</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>dig_or_inspect_choices</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>found_choices</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>nothing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>found_choices</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>goanna</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Goanna</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>found_choices</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>bluetongue</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Bluetongue</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>found_choices</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>king_brown</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>King Brown</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>found_choices</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Other</t>
         </is>
       </c>
     </row>

</xml_diff>